<commit_message>
Fix paginacion VTEX: leer todas las paginas segun recordsFiltered
No cortar cuando nuevos==0 porque paginas intermedias pueden no tener
aceite de oliva pero paginas siguientes si. Ahora se leen las 4 paginas
completas de Disco/Jumbo/Vea.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aceites_oliva_tracker.xlsx
+++ b/aceites_oliva_tracker.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H362"/>
+  <dimension ref="A1:H359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -3353,23 +3353,23 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Filippo Berio</t>
+          <t>Familia Zuccardi</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
+          <t>Aceite Oliva Genovesa Zuccardi 250 Ml</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>37950</v>
+        <v>16850</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" s="3" t="n">
-        <v>75900</v>
+        <v>67400</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
@@ -3385,23 +3385,23 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Familia Zuccardi</t>
+          <t>Filippo Berio</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Aceite Oliva Genovesa Zuccardi 250 Ml</t>
+          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>16850</v>
+        <v>37950</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" s="3" t="n">
-        <v>67400</v>
+        <v>75900</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
@@ -3615,29 +3615,27 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Pisi</t>
+          <t>Filippo Berio</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
+          <t>Aceite De Oliva Filippo Berio Extra Virgen 250 Ml</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>250</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>9180</v>
-      </c>
-      <c r="F97" s="3" t="n">
-        <v>10800</v>
-      </c>
+        <v>21150</v>
+      </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" s="3" t="n">
-        <v>36720</v>
+        <v>84600</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -3649,27 +3647,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Filippo Berio</t>
+          <t>Pisi</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Filippo Berio Extra Virgen 250 Ml</t>
+          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>250</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>21150</v>
-      </c>
-      <c r="F98" t="inlineStr"/>
+        <v>9180</v>
+      </c>
+      <c r="F98" s="3" t="n">
+        <v>10800</v>
+      </c>
       <c r="G98" s="3" t="n">
-        <v>84600</v>
+        <v>36720</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -5339,23 +5339,23 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Monini</t>
+          <t>Familia Zuccardi</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Monini Extra Virgen Delicato 500 Ml</t>
+          <t>Aceite Oliva Picual Zuccardi 500 Ml</t>
         </is>
       </c>
       <c r="D149" t="n">
         <v>500</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>24350</v>
+        <v>28850</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" s="3" t="n">
-        <v>48700</v>
+        <v>57700</v>
       </c>
       <c r="H149" t="inlineStr">
         <is>
@@ -5371,23 +5371,23 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Familia Zuccardi</t>
+          <t>Monini</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Aceite Oliva Picual Zuccardi 500 Ml</t>
+          <t>Aceite De Oliva Monini Extra Virgen Delicato 500 Ml</t>
         </is>
       </c>
       <c r="D150" t="n">
         <v>500</v>
       </c>
       <c r="E150" s="3" t="n">
-        <v>28850</v>
+        <v>24350</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" s="3" t="n">
-        <v>57700</v>
+        <v>48700</v>
       </c>
       <c r="H150" t="inlineStr">
         <is>
@@ -5663,23 +5663,23 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>La Toscana</t>
+          <t>Filippo Berio</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Con Ají Picante La Toscana 250 Ml</t>
+          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>14250</v>
+        <v>37950</v>
       </c>
       <c r="F159" t="inlineStr"/>
       <c r="G159" s="3" t="n">
-        <v>57000</v>
+        <v>75900</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
@@ -5695,23 +5695,23 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Filippo Berio</t>
+          <t>La Toscana</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
+          <t>Aceite De Oliva Extra Virgen Con Ají Picante La Toscana 250 Ml</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>37950</v>
+        <v>14250</v>
       </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" s="3" t="n">
-        <v>75900</v>
+        <v>57000</v>
       </c>
       <c r="H160" t="inlineStr">
         <is>
@@ -6695,25 +6695,25 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>Pisi</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Clasica Oliovita 1 L</t>
+          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="E190" s="3" t="n">
-        <v>34255</v>
+        <v>8882</v>
       </c>
       <c r="F190" s="3" t="n">
-        <v>40300</v>
+        <v>10450</v>
       </c>
       <c r="G190" s="3" t="n">
-        <v>34255</v>
+        <v>35530</v>
       </c>
       <c r="H190" t="inlineStr">
         <is>
@@ -6729,25 +6729,25 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Pisi</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
+          <t>Aceite De Oliva Extra Virgen Mediterraneo Oliovita 500 Ml</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="E191" s="3" t="n">
-        <v>8882</v>
+        <v>17552</v>
       </c>
       <c r="F191" s="3" t="n">
-        <v>10450</v>
+        <v>20650</v>
       </c>
       <c r="G191" s="3" t="n">
-        <v>35530</v>
+        <v>35105</v>
       </c>
       <c r="H191" t="inlineStr">
         <is>
@@ -6768,20 +6768,20 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Mediterraneo Oliovita 500 Ml</t>
+          <t>Aceite De Oliva Clasica Oliovita 1 L</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="E192" s="3" t="n">
-        <v>17552</v>
+        <v>34255</v>
       </c>
       <c r="F192" s="3" t="n">
-        <v>20650</v>
+        <v>40300</v>
       </c>
       <c r="G192" s="3" t="n">
-        <v>35105</v>
+        <v>34255</v>
       </c>
       <c r="H192" t="inlineStr">
         <is>
@@ -6931,29 +6931,27 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>Zuelo</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Oliovita Changlot 500 Ml</t>
+          <t>Aceite De Oliva Zuelo Extra Virgen Clásico 500 Ml</t>
         </is>
       </c>
       <c r="D197" t="n">
         <v>500</v>
       </c>
       <c r="E197" s="3" t="n">
-        <v>16830</v>
-      </c>
-      <c r="F197" s="3" t="n">
-        <v>19800</v>
-      </c>
+        <v>21050</v>
+      </c>
+      <c r="F197" t="inlineStr"/>
       <c r="G197" s="3" t="n">
-        <v>33660</v>
+        <v>42100</v>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -6965,27 +6963,29 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Zuelo</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Zuelo Extra Virgen Clásico 500 Ml</t>
+          <t>Aceite De Oliva Oliovita Changlot 500 Ml</t>
         </is>
       </c>
       <c r="D198" t="n">
         <v>500</v>
       </c>
       <c r="E198" s="3" t="n">
-        <v>21050</v>
-      </c>
-      <c r="F198" t="inlineStr"/>
+        <v>16830</v>
+      </c>
+      <c r="F198" s="3" t="n">
+        <v>19800</v>
+      </c>
       <c r="G198" s="3" t="n">
-        <v>42100</v>
+        <v>33660</v>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -12181,104 +12181,8 @@
         </is>
       </c>
     </row>
-    <row r="360">
-      <c r="A360" t="inlineStr">
-        <is>
-          <t>La Anonima</t>
-        </is>
-      </c>
-      <c r="B360" t="inlineStr">
-        <is>
-          <t>Familia Zuccardi</t>
-        </is>
-      </c>
-      <c r="C360" t="inlineStr">
-        <is>
-          <t>Aceite de Oliva Picual Vidrio Zuccardi x 500 cc.</t>
-        </is>
-      </c>
-      <c r="D360" t="n">
-        <v>500</v>
-      </c>
-      <c r="E360" s="3" t="n">
-        <v>29950</v>
-      </c>
-      <c r="F360" t="inlineStr"/>
-      <c r="G360" s="3" t="n">
-        <v>59900</v>
-      </c>
-      <c r="H360" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" t="inlineStr">
-        <is>
-          <t>La Anonima</t>
-        </is>
-      </c>
-      <c r="B361" t="inlineStr">
-        <is>
-          <t>Familia Zuccardi</t>
-        </is>
-      </c>
-      <c r="C361" t="inlineStr">
-        <is>
-          <t>Aceite de Oliva Coratina Vidrio Zuccardi x 500 cc.</t>
-        </is>
-      </c>
-      <c r="D361" t="n">
-        <v>500</v>
-      </c>
-      <c r="E361" s="3" t="n">
-        <v>29950</v>
-      </c>
-      <c r="F361" t="inlineStr"/>
-      <c r="G361" s="3" t="n">
-        <v>59900</v>
-      </c>
-      <c r="H361" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" t="inlineStr">
-        <is>
-          <t>La Anonima</t>
-        </is>
-      </c>
-      <c r="B362" t="inlineStr">
-        <is>
-          <t>Quesitos</t>
-        </is>
-      </c>
-      <c r="C362" t="inlineStr">
-        <is>
-          <t>Quesitos en Aceite de Oliva Familia Weiss x 100 g.</t>
-        </is>
-      </c>
-      <c r="D362" t="n">
-        <v>100</v>
-      </c>
-      <c r="E362" s="3" t="n">
-        <v>8900</v>
-      </c>
-      <c r="F362" t="inlineStr"/>
-      <c r="G362" s="3" t="n">
-        <v>89000</v>
-      </c>
-      <c r="H362" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="H4:H362">
+  <conditionalFormatting sqref="H4:H359">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Sí"</formula>
     </cfRule>
@@ -12296,7 +12200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1016"/>
+  <dimension ref="A1:K1013"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51015,23 +50919,23 @@
       </c>
       <c r="E851" t="inlineStr">
         <is>
-          <t>Monini</t>
+          <t>Familia Zuccardi</t>
         </is>
       </c>
       <c r="F851" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Monini Extra Virgen Delicato 500 Ml</t>
+          <t>Aceite Oliva Picual Zuccardi 500 Ml</t>
         </is>
       </c>
       <c r="G851" t="n">
         <v>500</v>
       </c>
       <c r="H851" s="3" t="n">
-        <v>24350</v>
+        <v>28850</v>
       </c>
       <c r="I851" t="inlineStr"/>
       <c r="J851" s="3" t="n">
-        <v>48700</v>
+        <v>57700</v>
       </c>
       <c r="K851" t="inlineStr">
         <is>
@@ -51060,23 +50964,23 @@
       </c>
       <c r="E852" t="inlineStr">
         <is>
-          <t>Familia Zuccardi</t>
+          <t>Monini</t>
         </is>
       </c>
       <c r="F852" t="inlineStr">
         <is>
-          <t>Aceite Oliva Picual Zuccardi 500 Ml</t>
+          <t>Aceite De Oliva Monini Extra Virgen Delicato 500 Ml</t>
         </is>
       </c>
       <c r="G852" t="n">
         <v>500</v>
       </c>
       <c r="H852" s="3" t="n">
-        <v>28850</v>
+        <v>24350</v>
       </c>
       <c r="I852" t="inlineStr"/>
       <c r="J852" s="3" t="n">
-        <v>57700</v>
+        <v>48700</v>
       </c>
       <c r="K852" t="inlineStr">
         <is>
@@ -51469,23 +51373,23 @@
       </c>
       <c r="E861" t="inlineStr">
         <is>
-          <t>La Toscana</t>
+          <t>Filippo Berio</t>
         </is>
       </c>
       <c r="F861" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Con Ají Picante La Toscana 250 Ml</t>
+          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
         </is>
       </c>
       <c r="G861" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H861" s="3" t="n">
-        <v>14250</v>
+        <v>37950</v>
       </c>
       <c r="I861" t="inlineStr"/>
       <c r="J861" s="3" t="n">
-        <v>57000</v>
+        <v>75900</v>
       </c>
       <c r="K861" t="inlineStr">
         <is>
@@ -51514,23 +51418,23 @@
       </c>
       <c r="E862" t="inlineStr">
         <is>
-          <t>Filippo Berio</t>
+          <t>La Toscana</t>
         </is>
       </c>
       <c r="F862" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
+          <t>Aceite De Oliva Extra Virgen Con Ají Picante La Toscana 250 Ml</t>
         </is>
       </c>
       <c r="G862" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H862" s="3" t="n">
-        <v>37950</v>
+        <v>14250</v>
       </c>
       <c r="I862" t="inlineStr"/>
       <c r="J862" s="3" t="n">
-        <v>75900</v>
+        <v>57000</v>
       </c>
       <c r="K862" t="inlineStr">
         <is>
@@ -54094,23 +53998,23 @@
       </c>
       <c r="E918" t="inlineStr">
         <is>
-          <t>Filippo Berio</t>
+          <t>Familia Zuccardi</t>
         </is>
       </c>
       <c r="F918" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
+          <t>Aceite Oliva Genovesa Zuccardi 250 Ml</t>
         </is>
       </c>
       <c r="G918" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H918" s="3" t="n">
-        <v>37950</v>
+        <v>16850</v>
       </c>
       <c r="I918" t="inlineStr"/>
       <c r="J918" s="3" t="n">
-        <v>75900</v>
+        <v>67400</v>
       </c>
       <c r="K918" t="inlineStr">
         <is>
@@ -54139,23 +54043,23 @@
       </c>
       <c r="E919" t="inlineStr">
         <is>
-          <t>Familia Zuccardi</t>
+          <t>Filippo Berio</t>
         </is>
       </c>
       <c r="F919" t="inlineStr">
         <is>
-          <t>Aceite Oliva Genovesa Zuccardi 250 Ml</t>
+          <t>Aceite De Oliva Filippo Berio Extra Virgen 500 Ml</t>
         </is>
       </c>
       <c r="G919" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H919" s="3" t="n">
-        <v>16850</v>
+        <v>37950</v>
       </c>
       <c r="I919" t="inlineStr"/>
       <c r="J919" s="3" t="n">
-        <v>67400</v>
+        <v>75900</v>
       </c>
       <c r="K919" t="inlineStr">
         <is>
@@ -54460,29 +54364,27 @@
       </c>
       <c r="E926" t="inlineStr">
         <is>
-          <t>Pisi</t>
+          <t>Filippo Berio</t>
         </is>
       </c>
       <c r="F926" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
+          <t>Aceite De Oliva Filippo Berio Extra Virgen 250 Ml</t>
         </is>
       </c>
       <c r="G926" t="n">
         <v>250</v>
       </c>
       <c r="H926" s="3" t="n">
-        <v>9180</v>
-      </c>
-      <c r="I926" s="3" t="n">
-        <v>10800</v>
-      </c>
+        <v>21150</v>
+      </c>
+      <c r="I926" t="inlineStr"/>
       <c r="J926" s="3" t="n">
-        <v>36720</v>
+        <v>84600</v>
       </c>
       <c r="K926" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -54507,27 +54409,29 @@
       </c>
       <c r="E927" t="inlineStr">
         <is>
-          <t>Filippo Berio</t>
+          <t>Pisi</t>
         </is>
       </c>
       <c r="F927" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Filippo Berio Extra Virgen 250 Ml</t>
+          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
         </is>
       </c>
       <c r="G927" t="n">
         <v>250</v>
       </c>
       <c r="H927" s="3" t="n">
-        <v>21150</v>
-      </c>
-      <c r="I927" t="inlineStr"/>
+        <v>9180</v>
+      </c>
+      <c r="I927" s="3" t="n">
+        <v>10800</v>
+      </c>
       <c r="J927" s="3" t="n">
-        <v>84600</v>
+        <v>36720</v>
       </c>
       <c r="K927" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -56635,32 +56539,34 @@
       </c>
       <c r="D974" t="inlineStr">
         <is>
-          <t>La Anonima</t>
+          <t>Vea</t>
         </is>
       </c>
       <c r="E974" t="inlineStr">
         <is>
-          <t>Familia Zuccardi</t>
+          <t>Cocinero</t>
         </is>
       </c>
       <c r="F974" t="inlineStr">
         <is>
-          <t>Aceite de Oliva Picual Vidrio Zuccardi x 500 cc.</t>
+          <t>Aceite Oliva Extra Virgen Intenso Cocinero 500 Ml</t>
         </is>
       </c>
       <c r="G974" t="n">
         <v>500</v>
       </c>
       <c r="H974" s="3" t="n">
-        <v>29950</v>
-      </c>
-      <c r="I974" t="inlineStr"/>
+        <v>11985</v>
+      </c>
+      <c r="I974" s="3" t="n">
+        <v>14100</v>
+      </c>
       <c r="J974" s="3" t="n">
-        <v>59900</v>
+        <v>23970</v>
       </c>
       <c r="K974" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -56680,32 +56586,34 @@
       </c>
       <c r="D975" t="inlineStr">
         <is>
-          <t>La Anonima</t>
+          <t>Vea</t>
         </is>
       </c>
       <c r="E975" t="inlineStr">
         <is>
-          <t>Familia Zuccardi</t>
+          <t>Cocinero</t>
         </is>
       </c>
       <c r="F975" t="inlineStr">
         <is>
-          <t>Aceite de Oliva Coratina Vidrio Zuccardi x 500 cc.</t>
+          <t>Aceite Oliva Extra Virgen Suave Cocinero 500 Ml</t>
         </is>
       </c>
       <c r="G975" t="n">
         <v>500</v>
       </c>
       <c r="H975" s="3" t="n">
-        <v>29950</v>
-      </c>
-      <c r="I975" t="inlineStr"/>
+        <v>11985</v>
+      </c>
+      <c r="I975" s="3" t="n">
+        <v>14100</v>
+      </c>
       <c r="J975" s="3" t="n">
-        <v>59900</v>
+        <v>23970</v>
       </c>
       <c r="K975" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -56725,32 +56633,34 @@
       </c>
       <c r="D976" t="inlineStr">
         <is>
-          <t>La Anonima</t>
+          <t>Vea</t>
         </is>
       </c>
       <c r="E976" t="inlineStr">
         <is>
-          <t>Quesitos</t>
+          <t>Cousine &amp; Co</t>
         </is>
       </c>
       <c r="F976" t="inlineStr">
         <is>
-          <t>Quesitos en Aceite de Oliva Familia Weiss x 100 g.</t>
+          <t>Aceite De Oliva Virgen 500 Ml Cuisine And Co</t>
         </is>
       </c>
       <c r="G976" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H976" s="3" t="n">
-        <v>8900</v>
-      </c>
-      <c r="I976" t="inlineStr"/>
+        <v>8274</v>
+      </c>
+      <c r="I976" s="3" t="n">
+        <v>12730</v>
+      </c>
       <c r="J976" s="3" t="n">
-        <v>89000</v>
+        <v>16549</v>
       </c>
       <c r="K976" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -56775,25 +56685,25 @@
       </c>
       <c r="E977" t="inlineStr">
         <is>
-          <t>Cocinero</t>
+          <t>Pisi</t>
         </is>
       </c>
       <c r="F977" t="inlineStr">
         <is>
-          <t>Aceite Oliva Extra Virgen Intenso Cocinero 500 Ml</t>
+          <t>Aceite De Oliva Extra Virgen X 500 Ml Pisi</t>
         </is>
       </c>
       <c r="G977" t="n">
         <v>500</v>
       </c>
       <c r="H977" s="3" t="n">
-        <v>11985</v>
+        <v>13685</v>
       </c>
       <c r="I977" s="3" t="n">
-        <v>14100</v>
+        <v>16100</v>
       </c>
       <c r="J977" s="3" t="n">
-        <v>23970</v>
+        <v>27370</v>
       </c>
       <c r="K977" t="inlineStr">
         <is>
@@ -56827,20 +56737,20 @@
       </c>
       <c r="F978" t="inlineStr">
         <is>
-          <t>Aceite Oliva Extra Virgen Suave Cocinero 500 Ml</t>
+          <t>Aceite De Oliva Cocinero Puro X500cc</t>
         </is>
       </c>
       <c r="G978" t="n">
         <v>500</v>
       </c>
       <c r="H978" s="3" t="n">
-        <v>11985</v>
+        <v>10242</v>
       </c>
       <c r="I978" s="3" t="n">
-        <v>14100</v>
+        <v>12050</v>
       </c>
       <c r="J978" s="3" t="n">
-        <v>23970</v>
+        <v>20485</v>
       </c>
       <c r="K978" t="inlineStr">
         <is>
@@ -56869,25 +56779,25 @@
       </c>
       <c r="E979" t="inlineStr">
         <is>
-          <t>Cousine &amp; Co</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="F979" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Virgen 500 Ml Cuisine And Co</t>
+          <t>Aceite De Oliva Oliovita Extra Virgen Clásico 500 Ml</t>
         </is>
       </c>
       <c r="G979" t="n">
         <v>500</v>
       </c>
       <c r="H979" s="3" t="n">
-        <v>8274</v>
+        <v>16532</v>
       </c>
       <c r="I979" s="3" t="n">
-        <v>12730</v>
+        <v>19450</v>
       </c>
       <c r="J979" s="3" t="n">
-        <v>16549</v>
+        <v>33065</v>
       </c>
       <c r="K979" t="inlineStr">
         <is>
@@ -56916,25 +56826,25 @@
       </c>
       <c r="E980" t="inlineStr">
         <is>
-          <t>Pisi</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="F980" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen X 500 Ml Pisi</t>
+          <t>Aceite De Oliva Mediterráneo Oliovita 500 Ml</t>
         </is>
       </c>
       <c r="G980" t="n">
         <v>500</v>
       </c>
       <c r="H980" s="3" t="n">
-        <v>13685</v>
+        <v>12028</v>
       </c>
       <c r="I980" s="3" t="n">
-        <v>16100</v>
+        <v>14150</v>
       </c>
       <c r="J980" s="3" t="n">
-        <v>27370</v>
+        <v>24055</v>
       </c>
       <c r="K980" t="inlineStr">
         <is>
@@ -56963,25 +56873,25 @@
       </c>
       <c r="E981" t="inlineStr">
         <is>
-          <t>Cocinero</t>
+          <t>Natura</t>
         </is>
       </c>
       <c r="F981" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Cocinero Puro X500cc</t>
+          <t>Aceite Natura Oliva Andino 500 Cc</t>
         </is>
       </c>
       <c r="G981" t="n">
         <v>500</v>
       </c>
       <c r="H981" s="3" t="n">
-        <v>10242</v>
+        <v>15428</v>
       </c>
       <c r="I981" s="3" t="n">
-        <v>12050</v>
+        <v>18150</v>
       </c>
       <c r="J981" s="3" t="n">
-        <v>20485</v>
+        <v>30855</v>
       </c>
       <c r="K981" t="inlineStr">
         <is>
@@ -57010,25 +56920,25 @@
       </c>
       <c r="E982" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>Nucete</t>
         </is>
       </c>
       <c r="F982" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Oliovita Extra Virgen Clásico 500 Ml</t>
+          <t>Aceite De Oliva Virgen Nucete Lata 500 Ml</t>
         </is>
       </c>
       <c r="G982" t="n">
         <v>500</v>
       </c>
       <c r="H982" s="3" t="n">
-        <v>16532</v>
+        <v>14068</v>
       </c>
       <c r="I982" s="3" t="n">
-        <v>19450</v>
+        <v>16550</v>
       </c>
       <c r="J982" s="3" t="n">
-        <v>33065</v>
+        <v>28135</v>
       </c>
       <c r="K982" t="inlineStr">
         <is>
@@ -57057,25 +56967,25 @@
       </c>
       <c r="E983" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>Nucete</t>
         </is>
       </c>
       <c r="F983" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Mediterráneo Oliovita 500 Ml</t>
+          <t>Aceite De Oliva Extra Virgen 2000 Ml Nucete</t>
         </is>
       </c>
       <c r="G983" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="H983" s="3" t="n">
-        <v>12028</v>
+        <v>39695</v>
       </c>
       <c r="I983" s="3" t="n">
-        <v>14150</v>
+        <v>46700</v>
       </c>
       <c r="J983" s="3" t="n">
-        <v>24055</v>
+        <v>19848</v>
       </c>
       <c r="K983" t="inlineStr">
         <is>
@@ -57104,25 +57014,25 @@
       </c>
       <c r="E984" t="inlineStr">
         <is>
-          <t>Natura</t>
+          <t>Cocinero</t>
         </is>
       </c>
       <c r="F984" t="inlineStr">
         <is>
-          <t>Aceite Natura Oliva Andino 500 Cc</t>
+          <t>Aceite De Oliva Cocinero Extra Virgen X500cc</t>
         </is>
       </c>
       <c r="G984" t="n">
         <v>500</v>
       </c>
       <c r="H984" s="3" t="n">
-        <v>15428</v>
+        <v>11985</v>
       </c>
       <c r="I984" s="3" t="n">
-        <v>18150</v>
+        <v>14100</v>
       </c>
       <c r="J984" s="3" t="n">
-        <v>30855</v>
+        <v>23970</v>
       </c>
       <c r="K984" t="inlineStr">
         <is>
@@ -57151,25 +57061,25 @@
       </c>
       <c r="E985" t="inlineStr">
         <is>
-          <t>Nucete</t>
+          <t>Natura</t>
         </is>
       </c>
       <c r="F985" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Virgen Nucete Lata 500 Ml</t>
+          <t>Aceite Natura Oliva Suave Bivarietal - 500 Ml</t>
         </is>
       </c>
       <c r="G985" t="n">
         <v>500</v>
       </c>
       <c r="H985" s="3" t="n">
-        <v>14068</v>
+        <v>12325</v>
       </c>
       <c r="I985" s="3" t="n">
-        <v>16550</v>
+        <v>14500</v>
       </c>
       <c r="J985" s="3" t="n">
-        <v>28135</v>
+        <v>24650</v>
       </c>
       <c r="K985" t="inlineStr">
         <is>
@@ -57203,20 +57113,20 @@
       </c>
       <c r="F986" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen 2000 Ml Nucete</t>
+          <t>Aceite De Oliva Nucete Extra Virgen Suave 500 Ml</t>
         </is>
       </c>
       <c r="G986" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="H986" s="3" t="n">
-        <v>39695</v>
+        <v>12665</v>
       </c>
       <c r="I986" s="3" t="n">
-        <v>46700</v>
+        <v>14900</v>
       </c>
       <c r="J986" s="3" t="n">
-        <v>19848</v>
+        <v>25330</v>
       </c>
       <c r="K986" t="inlineStr">
         <is>
@@ -57250,20 +57160,20 @@
       </c>
       <c r="F987" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Cocinero Extra Virgen X500cc</t>
+          <t>Aceite De Oliva Cocinero Extra Virgen X1l</t>
         </is>
       </c>
       <c r="G987" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="H987" s="3" t="n">
-        <v>11985</v>
+        <v>22865</v>
       </c>
       <c r="I987" s="3" t="n">
-        <v>14100</v>
+        <v>26900</v>
       </c>
       <c r="J987" s="3" t="n">
-        <v>23970</v>
+        <v>22865</v>
       </c>
       <c r="K987" t="inlineStr">
         <is>
@@ -57292,25 +57202,25 @@
       </c>
       <c r="E988" t="inlineStr">
         <is>
-          <t>Natura</t>
+          <t>Pisi</t>
         </is>
       </c>
       <c r="F988" t="inlineStr">
         <is>
-          <t>Aceite Natura Oliva Suave Bivarietal - 500 Ml</t>
+          <t>Aceite De Oliva 2 Lts Pisi</t>
         </is>
       </c>
       <c r="G988" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="H988" s="3" t="n">
-        <v>12325</v>
+        <v>34765</v>
       </c>
       <c r="I988" s="3" t="n">
-        <v>14500</v>
+        <v>40900</v>
       </c>
       <c r="J988" s="3" t="n">
-        <v>24650</v>
+        <v>17382</v>
       </c>
       <c r="K988" t="inlineStr">
         <is>
@@ -57339,25 +57249,25 @@
       </c>
       <c r="E989" t="inlineStr">
         <is>
-          <t>Nucete</t>
+          <t>Cousine &amp; Co</t>
         </is>
       </c>
       <c r="F989" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Nucete Extra Virgen Suave 500 Ml</t>
+          <t>Aceite De Oliva Extra Virgen 500 Ml Cuisine &amp; Co</t>
         </is>
       </c>
       <c r="G989" t="n">
         <v>500</v>
       </c>
       <c r="H989" s="3" t="n">
-        <v>12665</v>
+        <v>10465</v>
       </c>
       <c r="I989" s="3" t="n">
-        <v>14900</v>
+        <v>16100</v>
       </c>
       <c r="J989" s="3" t="n">
-        <v>25330</v>
+        <v>20930</v>
       </c>
       <c r="K989" t="inlineStr">
         <is>
@@ -57386,29 +57296,27 @@
       </c>
       <c r="E990" t="inlineStr">
         <is>
-          <t>Cocinero</t>
+          <t>Laur</t>
         </is>
       </c>
       <c r="F990" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Cocinero Extra Virgen X1l</t>
+          <t>Aceite Oliva Laur Blend Terroir Lata X500cc</t>
         </is>
       </c>
       <c r="G990" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="H990" s="3" t="n">
-        <v>22865</v>
-      </c>
-      <c r="I990" s="3" t="n">
-        <v>26900</v>
-      </c>
+        <v>16200</v>
+      </c>
+      <c r="I990" t="inlineStr"/>
       <c r="J990" s="3" t="n">
-        <v>22865</v>
+        <v>32400</v>
       </c>
       <c r="K990" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -57433,29 +57341,27 @@
       </c>
       <c r="E991" t="inlineStr">
         <is>
-          <t>Pisi</t>
+          <t>La Toscana</t>
         </is>
       </c>
       <c r="F991" t="inlineStr">
         <is>
-          <t>Aceite De Oliva 2 Lts Pisi</t>
+          <t>Aceite De Oliva La Toscana Extra Virgen 250 Ml</t>
         </is>
       </c>
       <c r="G991" t="n">
-        <v>2000</v>
+        <v>250</v>
       </c>
       <c r="H991" s="3" t="n">
-        <v>34765</v>
-      </c>
-      <c r="I991" s="3" t="n">
-        <v>40900</v>
-      </c>
+        <v>9450</v>
+      </c>
+      <c r="I991" t="inlineStr"/>
       <c r="J991" s="3" t="n">
-        <v>17382</v>
+        <v>37800</v>
       </c>
       <c r="K991" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -57485,20 +57391,20 @@
       </c>
       <c r="F992" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen 500 Ml Cuisine &amp; Co</t>
+          <t>Aceite De Oliva Extra Virgen 250 Ml Cuisine &amp; Co</t>
         </is>
       </c>
       <c r="G992" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H992" s="3" t="n">
-        <v>10465</v>
+        <v>7520</v>
       </c>
       <c r="I992" s="3" t="n">
-        <v>16100</v>
+        <v>11570</v>
       </c>
       <c r="J992" s="3" t="n">
-        <v>20930</v>
+        <v>30082</v>
       </c>
       <c r="K992" t="inlineStr">
         <is>
@@ -57527,27 +57433,29 @@
       </c>
       <c r="E993" t="inlineStr">
         <is>
-          <t>Laur</t>
+          <t>Natura</t>
         </is>
       </c>
       <c r="F993" t="inlineStr">
         <is>
-          <t>Aceite Oliva Laur Blend Terroir Lata X500cc</t>
+          <t>Aceite Natura Oliva Fuerte Trivar 500 Cc</t>
         </is>
       </c>
       <c r="G993" t="n">
         <v>500</v>
       </c>
       <c r="H993" s="3" t="n">
-        <v>16200</v>
-      </c>
-      <c r="I993" t="inlineStr"/>
+        <v>12325</v>
+      </c>
+      <c r="I993" s="3" t="n">
+        <v>14500</v>
+      </c>
       <c r="J993" s="3" t="n">
-        <v>32400</v>
+        <v>24650</v>
       </c>
       <c r="K993" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -57572,24 +57480,24 @@
       </c>
       <c r="E994" t="inlineStr">
         <is>
-          <t>La Toscana</t>
+          <t>Pisi</t>
         </is>
       </c>
       <c r="F994" t="inlineStr">
         <is>
-          <t>Aceite De Oliva La Toscana Extra Virgen 250 Ml</t>
-        </is>
-      </c>
-      <c r="G994" t="n">
-        <v>250</v>
+          <t>Aceite De Oliva Extra Virgen Pisi Premium</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>S/D</t>
+        </is>
       </c>
       <c r="H994" s="3" t="n">
-        <v>9450</v>
+        <v>21300</v>
       </c>
       <c r="I994" t="inlineStr"/>
-      <c r="J994" s="3" t="n">
-        <v>37800</v>
-      </c>
+      <c r="J994" t="inlineStr"/>
       <c r="K994" t="inlineStr">
         <is>
           <t>No</t>
@@ -57622,20 +57530,20 @@
       </c>
       <c r="F995" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen 250 Ml Cuisine &amp; Co</t>
+          <t>Aceite De Oliva Extra Virgen 500 Ml Cuisine &amp; Co</t>
         </is>
       </c>
       <c r="G995" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H995" s="3" t="n">
-        <v>7520</v>
+        <v>11940</v>
       </c>
       <c r="I995" s="3" t="n">
-        <v>11570</v>
+        <v>18370</v>
       </c>
       <c r="J995" s="3" t="n">
-        <v>30082</v>
+        <v>23881</v>
       </c>
       <c r="K995" t="inlineStr">
         <is>
@@ -57664,25 +57572,25 @@
       </c>
       <c r="E996" t="inlineStr">
         <is>
-          <t>Natura</t>
+          <t>Cocinero</t>
         </is>
       </c>
       <c r="F996" t="inlineStr">
         <is>
-          <t>Aceite Natura Oliva Fuerte Trivar 500 Cc</t>
+          <t>Aceite De Oliva Cocinero Puro X1l</t>
         </is>
       </c>
       <c r="G996" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="H996" s="3" t="n">
-        <v>12325</v>
+        <v>19422</v>
       </c>
       <c r="I996" s="3" t="n">
-        <v>14500</v>
+        <v>22850</v>
       </c>
       <c r="J996" s="3" t="n">
-        <v>24650</v>
+        <v>19422</v>
       </c>
       <c r="K996" t="inlineStr">
         <is>
@@ -57716,22 +57624,24 @@
       </c>
       <c r="F997" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Pisi Premium</t>
-        </is>
-      </c>
-      <c r="G997" t="inlineStr">
-        <is>
-          <t>S/D</t>
-        </is>
+          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
+        </is>
+      </c>
+      <c r="G997" t="n">
+        <v>250</v>
       </c>
       <c r="H997" s="3" t="n">
-        <v>21300</v>
-      </c>
-      <c r="I997" t="inlineStr"/>
-      <c r="J997" t="inlineStr"/>
+        <v>8882</v>
+      </c>
+      <c r="I997" s="3" t="n">
+        <v>10450</v>
+      </c>
+      <c r="J997" s="3" t="n">
+        <v>35530</v>
+      </c>
       <c r="K997" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -57756,25 +57666,25 @@
       </c>
       <c r="E998" t="inlineStr">
         <is>
-          <t>Cousine &amp; Co</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="F998" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen 500 Ml Cuisine &amp; Co</t>
+          <t>Aceite De Oliva Extra Virgen Mediterraneo Oliovita 500 Ml</t>
         </is>
       </c>
       <c r="G998" t="n">
         <v>500</v>
       </c>
       <c r="H998" s="3" t="n">
-        <v>11940</v>
+        <v>17552</v>
       </c>
       <c r="I998" s="3" t="n">
-        <v>18370</v>
+        <v>20650</v>
       </c>
       <c r="J998" s="3" t="n">
-        <v>23881</v>
+        <v>35105</v>
       </c>
       <c r="K998" t="inlineStr">
         <is>
@@ -57803,25 +57713,25 @@
       </c>
       <c r="E999" t="inlineStr">
         <is>
-          <t>Cocinero</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="F999" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Cocinero Puro X1l</t>
+          <t>Aceite De Oliva Clasica Oliovita 1 L</t>
         </is>
       </c>
       <c r="G999" t="n">
         <v>1000</v>
       </c>
       <c r="H999" s="3" t="n">
-        <v>19422</v>
+        <v>34255</v>
       </c>
       <c r="I999" s="3" t="n">
-        <v>22850</v>
+        <v>40300</v>
       </c>
       <c r="J999" s="3" t="n">
-        <v>19422</v>
+        <v>34255</v>
       </c>
       <c r="K999" t="inlineStr">
         <is>
@@ -57850,25 +57760,25 @@
       </c>
       <c r="E1000" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>La Toscana</t>
         </is>
       </c>
       <c r="F1000" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Clasica Oliovita 1 L</t>
+          <t>Aceite De Oliva La Toscana Extra Virgen 500 Ml</t>
         </is>
       </c>
       <c r="G1000" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="H1000" s="3" t="n">
-        <v>34255</v>
+        <v>15555</v>
       </c>
       <c r="I1000" s="3" t="n">
-        <v>40300</v>
+        <v>18300</v>
       </c>
       <c r="J1000" s="3" t="n">
-        <v>34255</v>
+        <v>31110</v>
       </c>
       <c r="K1000" t="inlineStr">
         <is>
@@ -57897,25 +57807,25 @@
       </c>
       <c r="E1001" t="inlineStr">
         <is>
-          <t>Pisi</t>
+          <t>Nucete</t>
         </is>
       </c>
       <c r="F1001" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Pisi   Bot 250 Cc.</t>
+          <t>Aceite De Oliva Nucete Extra Virgen Intenso 500 Ml</t>
         </is>
       </c>
       <c r="G1001" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="H1001" s="3" t="n">
-        <v>8882</v>
+        <v>13982</v>
       </c>
       <c r="I1001" s="3" t="n">
-        <v>10450</v>
+        <v>16450</v>
       </c>
       <c r="J1001" s="3" t="n">
-        <v>35530</v>
+        <v>27965</v>
       </c>
       <c r="K1001" t="inlineStr">
         <is>
@@ -57944,29 +57854,27 @@
       </c>
       <c r="E1002" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>Yancanello</t>
         </is>
       </c>
       <c r="F1002" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Mediterraneo Oliovita 500 Ml</t>
+          <t>Aceite De Oliva Yancanello Extra Virgen 1 L</t>
         </is>
       </c>
       <c r="G1002" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="H1002" s="3" t="n">
-        <v>17552</v>
-      </c>
-      <c r="I1002" s="3" t="n">
-        <v>20650</v>
-      </c>
+        <v>51100</v>
+      </c>
+      <c r="I1002" t="inlineStr"/>
       <c r="J1002" s="3" t="n">
-        <v>35105</v>
+        <v>51100</v>
       </c>
       <c r="K1002" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -57991,25 +57899,25 @@
       </c>
       <c r="E1003" t="inlineStr">
         <is>
-          <t>La Toscana</t>
+          <t>Cousine &amp; Co</t>
         </is>
       </c>
       <c r="F1003" t="inlineStr">
         <is>
-          <t>Aceite De Oliva La Toscana Extra Virgen 500 Ml</t>
+          <t>Aceite De Oliva Extra Virgen Cuisine And Co 1 L</t>
         </is>
       </c>
       <c r="G1003" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="H1003" s="3" t="n">
-        <v>15555</v>
+        <v>19728</v>
       </c>
       <c r="I1003" s="3" t="n">
-        <v>18300</v>
+        <v>30350</v>
       </c>
       <c r="J1003" s="3" t="n">
-        <v>31110</v>
+        <v>19728</v>
       </c>
       <c r="K1003" t="inlineStr">
         <is>
@@ -58038,29 +57946,27 @@
       </c>
       <c r="E1004" t="inlineStr">
         <is>
-          <t>Nucete</t>
+          <t>Zuelo</t>
         </is>
       </c>
       <c r="F1004" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Nucete Extra Virgen Intenso 500 Ml</t>
+          <t>Aceite De Oliva Zuelo Extra Virgen Clásico 500 Ml</t>
         </is>
       </c>
       <c r="G1004" t="n">
         <v>500</v>
       </c>
       <c r="H1004" s="3" t="n">
-        <v>13982</v>
-      </c>
-      <c r="I1004" s="3" t="n">
-        <v>16450</v>
-      </c>
+        <v>21050</v>
+      </c>
+      <c r="I1004" t="inlineStr"/>
       <c r="J1004" s="3" t="n">
-        <v>27965</v>
+        <v>42100</v>
       </c>
       <c r="K1004" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -58085,27 +57991,29 @@
       </c>
       <c r="E1005" t="inlineStr">
         <is>
-          <t>Yancanello</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="F1005" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Yancanello Extra Virgen 1 L</t>
+          <t>Aceite De Oliva Oliovita Changlot 500 Ml</t>
         </is>
       </c>
       <c r="G1005" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="H1005" s="3" t="n">
-        <v>51100</v>
-      </c>
-      <c r="I1005" t="inlineStr"/>
+        <v>16830</v>
+      </c>
+      <c r="I1005" s="3" t="n">
+        <v>19800</v>
+      </c>
       <c r="J1005" s="3" t="n">
-        <v>51100</v>
+        <v>33660</v>
       </c>
       <c r="K1005" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -58130,25 +58038,25 @@
       </c>
       <c r="E1006" t="inlineStr">
         <is>
-          <t>Cousine &amp; Co</t>
+          <t>Oliovita</t>
         </is>
       </c>
       <c r="F1006" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Extra Virgen Cuisine And Co 1 L</t>
+          <t>Aceite De Oliva Oliovita Extra Virgen Arbequina 500 Ml</t>
         </is>
       </c>
       <c r="G1006" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="H1006" s="3" t="n">
-        <v>19728</v>
+        <v>17085</v>
       </c>
       <c r="I1006" s="3" t="n">
-        <v>30350</v>
+        <v>20100</v>
       </c>
       <c r="J1006" s="3" t="n">
-        <v>19728</v>
+        <v>34170</v>
       </c>
       <c r="K1006" t="inlineStr">
         <is>
@@ -58182,24 +58090,22 @@
       </c>
       <c r="F1007" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Oliovita Changlot 500 Ml</t>
-        </is>
-      </c>
-      <c r="G1007" t="n">
-        <v>500</v>
+          <t>Aceite De Oliva Oliovita Coratina</t>
+        </is>
+      </c>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>S/D</t>
+        </is>
       </c>
       <c r="H1007" s="3" t="n">
-        <v>16830</v>
-      </c>
-      <c r="I1007" s="3" t="n">
-        <v>19800</v>
-      </c>
-      <c r="J1007" s="3" t="n">
-        <v>33660</v>
-      </c>
+        <v>22400</v>
+      </c>
+      <c r="I1007" t="inlineStr"/>
+      <c r="J1007" t="inlineStr"/>
       <c r="K1007" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -58224,27 +58130,29 @@
       </c>
       <c r="E1008" t="inlineStr">
         <is>
-          <t>Zuelo</t>
+          <t>Cousine &amp; Co</t>
         </is>
       </c>
       <c r="F1008" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Zuelo Extra Virgen Clásico 500 Ml</t>
+          <t>Aceite De Oliva Organico 250 Ml Cuisine &amp; Co</t>
         </is>
       </c>
       <c r="G1008" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H1008" s="3" t="n">
-        <v>21050</v>
-      </c>
-      <c r="I1008" t="inlineStr"/>
+        <v>8288</v>
+      </c>
+      <c r="I1008" s="3" t="n">
+        <v>12750</v>
+      </c>
       <c r="J1008" s="3" t="n">
-        <v>42100</v>
+        <v>33150</v>
       </c>
       <c r="K1008" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -58274,20 +58182,20 @@
       </c>
       <c r="F1009" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Oliovita Extra Virgen Arbequina 500 Ml</t>
+          <t>Aceite De Oliva Oliovita 1lt</t>
         </is>
       </c>
       <c r="G1009" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="H1009" s="3" t="n">
-        <v>17085</v>
+        <v>37782</v>
       </c>
       <c r="I1009" s="3" t="n">
-        <v>20100</v>
+        <v>44450</v>
       </c>
       <c r="J1009" s="3" t="n">
-        <v>34170</v>
+        <v>37782</v>
       </c>
       <c r="K1009" t="inlineStr">
         <is>
@@ -58316,27 +58224,29 @@
       </c>
       <c r="E1010" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>Cousine &amp; Co</t>
         </is>
       </c>
       <c r="F1010" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Oliovita Coratina</t>
-        </is>
-      </c>
-      <c r="G1010" t="inlineStr">
-        <is>
-          <t>S/D</t>
-        </is>
+          <t>Aceite De Oliva Organico 500 Ml Cuisine &amp; Co</t>
+        </is>
+      </c>
+      <c r="G1010" t="n">
+        <v>500</v>
       </c>
       <c r="H1010" s="3" t="n">
-        <v>22400</v>
-      </c>
-      <c r="I1010" t="inlineStr"/>
-      <c r="J1010" t="inlineStr"/>
+        <v>11278</v>
+      </c>
+      <c r="I1010" s="3" t="n">
+        <v>17350</v>
+      </c>
+      <c r="J1010" s="3" t="n">
+        <v>22555</v>
+      </c>
       <c r="K1010" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -58366,20 +58276,20 @@
       </c>
       <c r="F1011" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Organico 250 Ml Cuisine &amp; Co</t>
+          <t>Aceite De Oliva Extra Virgen 1 Lts Cuisine &amp; Co</t>
         </is>
       </c>
       <c r="G1011" t="n">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="H1011" s="3" t="n">
-        <v>8288</v>
+        <v>25571</v>
       </c>
       <c r="I1011" s="3" t="n">
-        <v>12750</v>
+        <v>39340</v>
       </c>
       <c r="J1011" s="3" t="n">
-        <v>33150</v>
+        <v>25571</v>
       </c>
       <c r="K1011" t="inlineStr">
         <is>
@@ -58408,29 +58318,27 @@
       </c>
       <c r="E1012" t="inlineStr">
         <is>
-          <t>Oliovita</t>
+          <t>Cousine &amp; Co</t>
         </is>
       </c>
       <c r="F1012" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Oliovita 1lt</t>
+          <t>Aceite Oliva Virgen Extra X 250 Ml Cuisine &amp; Co</t>
         </is>
       </c>
       <c r="G1012" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="H1012" s="3" t="n">
-        <v>37782</v>
-      </c>
-      <c r="I1012" s="3" t="n">
-        <v>44450</v>
-      </c>
+        <v>11900</v>
+      </c>
+      <c r="I1012" t="inlineStr"/>
       <c r="J1012" s="3" t="n">
-        <v>37782</v>
+        <v>47600</v>
       </c>
       <c r="K1012" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -58460,166 +58368,27 @@
       </c>
       <c r="F1013" t="inlineStr">
         <is>
-          <t>Aceite De Oliva Organico 500 Ml Cuisine &amp; Co</t>
+          <t>Aceite Oliva Virgen Extra X 500 Ml Cuisine &amp; Co</t>
         </is>
       </c>
       <c r="G1013" t="n">
         <v>500</v>
       </c>
       <c r="H1013" s="3" t="n">
-        <v>11278</v>
-      </c>
-      <c r="I1013" s="3" t="n">
-        <v>17350</v>
-      </c>
+        <v>21550</v>
+      </c>
+      <c r="I1013" t="inlineStr"/>
       <c r="J1013" s="3" t="n">
-        <v>22555</v>
+        <v>43100</v>
       </c>
       <c r="K1013" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="1014">
-      <c r="A1014" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="B1014" t="inlineStr">
-        <is>
-          <t>Marzo</t>
-        </is>
-      </c>
-      <c r="C1014" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D1014" t="inlineStr">
-        <is>
-          <t>Vea</t>
-        </is>
-      </c>
-      <c r="E1014" t="inlineStr">
-        <is>
-          <t>Cousine &amp; Co</t>
-        </is>
-      </c>
-      <c r="F1014" t="inlineStr">
-        <is>
-          <t>Aceite De Oliva Extra Virgen 1 Lts Cuisine &amp; Co</t>
-        </is>
-      </c>
-      <c r="G1014" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H1014" s="3" t="n">
-        <v>25571</v>
-      </c>
-      <c r="I1014" s="3" t="n">
-        <v>39340</v>
-      </c>
-      <c r="J1014" s="3" t="n">
-        <v>25571</v>
-      </c>
-      <c r="K1014" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="1015">
-      <c r="A1015" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="B1015" t="inlineStr">
-        <is>
-          <t>Marzo</t>
-        </is>
-      </c>
-      <c r="C1015" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D1015" t="inlineStr">
-        <is>
-          <t>Vea</t>
-        </is>
-      </c>
-      <c r="E1015" t="inlineStr">
-        <is>
-          <t>Cousine &amp; Co</t>
-        </is>
-      </c>
-      <c r="F1015" t="inlineStr">
-        <is>
-          <t>Aceite Oliva Virgen Extra X 250 Ml Cuisine &amp; Co</t>
-        </is>
-      </c>
-      <c r="G1015" t="n">
-        <v>250</v>
-      </c>
-      <c r="H1015" s="3" t="n">
-        <v>11900</v>
-      </c>
-      <c r="I1015" t="inlineStr"/>
-      <c r="J1015" s="3" t="n">
-        <v>47600</v>
-      </c>
-      <c r="K1015" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="1016">
-      <c r="A1016" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="B1016" t="inlineStr">
-        <is>
-          <t>Marzo</t>
-        </is>
-      </c>
-      <c r="C1016" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D1016" t="inlineStr">
-        <is>
-          <t>Vea</t>
-        </is>
-      </c>
-      <c r="E1016" t="inlineStr">
-        <is>
-          <t>Cousine &amp; Co</t>
-        </is>
-      </c>
-      <c r="F1016" t="inlineStr">
-        <is>
-          <t>Aceite Oliva Virgen Extra X 500 Ml Cuisine &amp; Co</t>
-        </is>
-      </c>
-      <c r="G1016" t="n">
-        <v>500</v>
-      </c>
-      <c r="H1016" s="3" t="n">
-        <v>21550</v>
-      </c>
-      <c r="I1016" t="inlineStr"/>
-      <c r="J1016" s="3" t="n">
-        <v>43100</v>
-      </c>
-      <c r="K1016" t="inlineStr">
-        <is>
           <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K2:K1016">
+  <conditionalFormatting sqref="K2:K1013">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Sí"</formula>
     </cfRule>
@@ -58637,7 +58406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K239"/>
+  <dimension ref="A1:K238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65069,21 +64838,21 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Quesitos</t>
+          <t>Rastrilla</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="D231" t="inlineStr"/>
       <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr"/>
+      <c r="F231" s="3" t="n">
+        <v>20500</v>
+      </c>
       <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr"/>
-      <c r="J231" s="3" t="n">
-        <v>8900</v>
-      </c>
+      <c r="J231" t="inlineStr"/>
       <c r="K231" t="inlineStr"/>
     </row>
     <row r="232">
@@ -65094,20 +64863,22 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Rastrilla</t>
+          <t>Vigil</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>500</v>
+        <v>120</v>
       </c>
       <c r="D232" t="inlineStr"/>
       <c r="E232" t="inlineStr"/>
-      <c r="F232" s="3" t="n">
-        <v>20500</v>
-      </c>
-      <c r="G232" t="inlineStr"/>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" s="3" t="n">
+        <v>9450</v>
+      </c>
       <c r="H232" t="inlineStr"/>
-      <c r="I232" t="inlineStr"/>
+      <c r="I232" s="3" t="n">
+        <v>9200</v>
+      </c>
       <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr"/>
     </row>
@@ -65119,21 +64890,21 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Vigil</t>
+          <t>Yancanello</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>120</v>
+        <v>500</v>
       </c>
       <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr"/>
       <c r="G233" s="3" t="n">
-        <v>9450</v>
+        <v>30800</v>
       </c>
       <c r="H233" t="inlineStr"/>
       <c r="I233" s="3" t="n">
-        <v>9200</v>
+        <v>29600</v>
       </c>
       <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr"/>
@@ -65150,20 +64921,20 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="D234" t="inlineStr"/>
       <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr"/>
       <c r="G234" s="3" t="n">
-        <v>30800</v>
+        <v>54850</v>
       </c>
       <c r="H234" t="inlineStr"/>
-      <c r="I234" s="3" t="n">
-        <v>29600</v>
-      </c>
+      <c r="I234" t="inlineStr"/>
       <c r="J234" t="inlineStr"/>
-      <c r="K234" t="inlineStr"/>
+      <c r="K234" s="3" t="n">
+        <v>51100</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -65173,24 +64944,26 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Yancanello</t>
+          <t>Ybarra</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="D235" t="inlineStr"/>
       <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
+      <c r="F235" s="3" t="n">
+        <v>31434</v>
+      </c>
       <c r="G235" s="3" t="n">
-        <v>54850</v>
+        <v>17750</v>
       </c>
       <c r="H235" t="inlineStr"/>
-      <c r="I235" t="inlineStr"/>
+      <c r="I235" s="3" t="n">
+        <v>17250</v>
+      </c>
       <c r="J235" t="inlineStr"/>
-      <c r="K235" s="3" t="n">
-        <v>51100</v>
-      </c>
+      <c r="K235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -65200,7 +64973,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Ybarra</t>
+          <t>Zuelo</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -65209,15 +64982,13 @@
       <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr"/>
       <c r="F236" s="3" t="n">
-        <v>31434</v>
+        <v>14926</v>
       </c>
       <c r="G236" s="3" t="n">
-        <v>17750</v>
+        <v>16150</v>
       </c>
       <c r="H236" t="inlineStr"/>
-      <c r="I236" s="3" t="n">
-        <v>17250</v>
-      </c>
+      <c r="I236" t="inlineStr"/>
       <c r="J236" t="inlineStr"/>
       <c r="K236" t="inlineStr"/>
     </row>
@@ -65233,20 +65004,28 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>250</v>
-      </c>
-      <c r="D237" t="inlineStr"/>
+        <v>500</v>
+      </c>
+      <c r="D237" s="3" t="n">
+        <v>20049</v>
+      </c>
       <c r="E237" t="inlineStr"/>
       <c r="F237" s="3" t="n">
-        <v>14926</v>
+        <v>20049</v>
       </c>
       <c r="G237" s="3" t="n">
-        <v>16150</v>
+        <v>22050</v>
       </c>
       <c r="H237" t="inlineStr"/>
-      <c r="I237" t="inlineStr"/>
-      <c r="J237" t="inlineStr"/>
-      <c r="K237" t="inlineStr"/>
+      <c r="I237" s="3" t="n">
+        <v>21650</v>
+      </c>
+      <c r="J237" s="3" t="n">
+        <v>20650</v>
+      </c>
+      <c r="K237" s="3" t="n">
+        <v>21050</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -65260,53 +65039,18 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>500</v>
-      </c>
-      <c r="D238" s="3" t="n">
-        <v>20049</v>
-      </c>
+        <v>2000</v>
+      </c>
+      <c r="D238" t="inlineStr"/>
       <c r="E238" t="inlineStr"/>
       <c r="F238" s="3" t="n">
-        <v>20049</v>
-      </c>
-      <c r="G238" s="3" t="n">
-        <v>22050</v>
-      </c>
+        <v>83283</v>
+      </c>
+      <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr"/>
-      <c r="I238" s="3" t="n">
-        <v>21650</v>
-      </c>
-      <c r="J238" s="3" t="n">
-        <v>20650</v>
-      </c>
-      <c r="K238" s="3" t="n">
-        <v>21050</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>Zuelo</t>
-        </is>
-      </c>
-      <c r="C239" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D239" t="inlineStr"/>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" s="3" t="n">
-        <v>83283</v>
-      </c>
-      <c r="G239" t="inlineStr"/>
-      <c r="H239" t="inlineStr"/>
-      <c r="I239" t="inlineStr"/>
-      <c r="J239" t="inlineStr"/>
-      <c r="K239" t="inlineStr"/>
+      <c r="I238" t="inlineStr"/>
+      <c r="J238" t="inlineStr"/>
+      <c r="K238" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>